<commit_message>
Add SAT Sonoscan workbench and activity tracking
</commit_message>
<xml_diff>
--- a/Rel Website/backend/templates/REL LTC Template.xlsx
+++ b/Rel Website/backend/templates/REL LTC Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amkor-my.sharepoint.com/personal/francisnino_villanueva_amkor_com/Documents/Documents/GitHub/Rel Request Process Flow/Rel Website/backend/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{55472A56-189D-460A-834D-19C0FE061C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B78F68D-4A9A-4534-B89D-92D23FB2DDF7}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{55472A56-189D-460A-834D-19C0FE061C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24C4256D-2630-42FA-B465-31E3D30E8790}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1350" yWindow="1950" windowWidth="27450" windowHeight="9990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1131,6 +1131,36 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1172,36 +1202,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -1304,202 +1304,11 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>117242</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>30873</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>318881</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>214724</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Rectangle 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A76155A2-70B2-4CA8-8A20-DF3B6EE63D92}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2416849" y="26728087"/>
-          <a:ext cx="201639" cy="183851"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="19050">
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-PH"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>133145</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>30874</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>334235</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>202924</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="Rectangle 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDFE29FD-AE8D-4F68-8194-EC60CB3A8E79}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2868181" y="26728088"/>
-          <a:ext cx="201090" cy="172050"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="19050">
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-PH"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>142874</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>35719</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>343964</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>207769</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="Rectangle 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3762D108-DDAC-4A68-BD66-2362739EBE63}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3313338" y="26732933"/>
-          <a:ext cx="201090" cy="172050"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="19050">
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-PH"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2195,46 +2004,46 @@
       <c r="T20" s="16"/>
     </row>
     <row r="21" spans="2:21" ht="120" customHeight="1">
-      <c r="B21" s="86"/>
-      <c r="C21" s="87"/>
-      <c r="D21" s="87"/>
-      <c r="E21" s="87"/>
-      <c r="F21" s="87"/>
-      <c r="G21" s="87"/>
-      <c r="H21" s="87"/>
-      <c r="I21" s="87"/>
-      <c r="J21" s="87"/>
-      <c r="K21" s="87"/>
-      <c r="L21" s="87"/>
-      <c r="M21" s="87"/>
-      <c r="N21" s="87"/>
-      <c r="O21" s="87"/>
-      <c r="P21" s="87"/>
-      <c r="Q21" s="87"/>
-      <c r="R21" s="87"/>
-      <c r="S21" s="87"/>
-      <c r="T21" s="88"/>
+      <c r="B21" s="96"/>
+      <c r="C21" s="97"/>
+      <c r="D21" s="97"/>
+      <c r="E21" s="97"/>
+      <c r="F21" s="97"/>
+      <c r="G21" s="97"/>
+      <c r="H21" s="97"/>
+      <c r="I21" s="97"/>
+      <c r="J21" s="97"/>
+      <c r="K21" s="97"/>
+      <c r="L21" s="97"/>
+      <c r="M21" s="97"/>
+      <c r="N21" s="97"/>
+      <c r="O21" s="97"/>
+      <c r="P21" s="97"/>
+      <c r="Q21" s="97"/>
+      <c r="R21" s="97"/>
+      <c r="S21" s="97"/>
+      <c r="T21" s="98"/>
     </row>
     <row r="22" spans="2:21" ht="60" customHeight="1">
-      <c r="B22" s="89"/>
-      <c r="C22" s="90"/>
-      <c r="D22" s="90"/>
-      <c r="E22" s="90"/>
-      <c r="F22" s="90"/>
-      <c r="G22" s="90"/>
-      <c r="H22" s="90"/>
-      <c r="I22" s="90"/>
-      <c r="J22" s="90"/>
-      <c r="K22" s="90"/>
-      <c r="L22" s="90"/>
-      <c r="M22" s="90"/>
-      <c r="N22" s="90"/>
-      <c r="O22" s="90"/>
-      <c r="P22" s="90"/>
-      <c r="Q22" s="90"/>
-      <c r="R22" s="90"/>
-      <c r="S22" s="90"/>
-      <c r="T22" s="91"/>
+      <c r="B22" s="99"/>
+      <c r="C22" s="100"/>
+      <c r="D22" s="100"/>
+      <c r="E22" s="100"/>
+      <c r="F22" s="100"/>
+      <c r="G22" s="100"/>
+      <c r="H22" s="100"/>
+      <c r="I22" s="100"/>
+      <c r="J22" s="100"/>
+      <c r="K22" s="100"/>
+      <c r="L22" s="100"/>
+      <c r="M22" s="100"/>
+      <c r="N22" s="100"/>
+      <c r="O22" s="100"/>
+      <c r="P22" s="100"/>
+      <c r="Q22" s="100"/>
+      <c r="R22" s="100"/>
+      <c r="S22" s="100"/>
+      <c r="T22" s="101"/>
     </row>
     <row r="23" spans="2:21" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="B23" s="12"/>
@@ -2287,10 +2096,10 @@
       <c r="C25" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="108" t="s">
+      <c r="D25" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="E25" s="109"/>
+      <c r="E25" s="87"/>
       <c r="F25" s="65" t="s">
         <v>28</v>
       </c>
@@ -2330,16 +2139,16 @@
       <c r="C26" s="76"/>
       <c r="D26" s="77"/>
       <c r="E26" s="78"/>
-      <c r="F26" s="97"/>
-      <c r="G26" s="99"/>
+      <c r="F26" s="107"/>
+      <c r="G26" s="109"/>
       <c r="H26" s="77"/>
       <c r="I26" s="78"/>
       <c r="J26" s="77"/>
       <c r="K26" s="79"/>
       <c r="L26" s="78"/>
-      <c r="M26" s="97"/>
-      <c r="N26" s="98"/>
-      <c r="O26" s="99"/>
+      <c r="M26" s="107"/>
+      <c r="N26" s="108"/>
+      <c r="O26" s="109"/>
       <c r="P26" s="76"/>
       <c r="Q26" s="76"/>
       <c r="R26" s="76"/>
@@ -2352,8 +2161,8 @@
       <c r="C27" s="76"/>
       <c r="D27" s="77"/>
       <c r="E27" s="78"/>
-      <c r="F27" s="97"/>
-      <c r="G27" s="99"/>
+      <c r="F27" s="107"/>
+      <c r="G27" s="109"/>
       <c r="H27" s="77"/>
       <c r="I27" s="78"/>
       <c r="J27" s="77"/>
@@ -2374,8 +2183,8 @@
       <c r="C28" s="76"/>
       <c r="D28" s="77"/>
       <c r="E28" s="78"/>
-      <c r="F28" s="97"/>
-      <c r="G28" s="99"/>
+      <c r="F28" s="107"/>
+      <c r="G28" s="109"/>
       <c r="H28" s="77"/>
       <c r="I28" s="78"/>
       <c r="J28" s="77"/>
@@ -2440,24 +2249,24 @@
       <c r="H32" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="I32" s="105" t="s">
+      <c r="I32" s="93" t="s">
         <v>42</v>
       </c>
-      <c r="J32" s="106"/>
-      <c r="K32" s="107"/>
-      <c r="L32" s="105" t="s">
+      <c r="J32" s="94"/>
+      <c r="K32" s="95"/>
+      <c r="L32" s="93" t="s">
         <v>43</v>
       </c>
-      <c r="M32" s="106"/>
-      <c r="N32" s="107"/>
-      <c r="O32" s="92" t="s">
+      <c r="M32" s="94"/>
+      <c r="N32" s="95"/>
+      <c r="O32" s="102" t="s">
         <v>44</v>
       </c>
-      <c r="P32" s="93"/>
-      <c r="Q32" s="92" t="s">
+      <c r="P32" s="103"/>
+      <c r="Q32" s="102" t="s">
         <v>45</v>
       </c>
-      <c r="R32" s="93"/>
+      <c r="R32" s="103"/>
       <c r="S32" s="27" t="s">
         <v>46</v>
       </c>
@@ -2468,10 +2277,10 @@
     <row r="33" spans="2:20" ht="30" customHeight="1">
       <c r="B33" s="5"/>
       <c r="C33" s="30"/>
-      <c r="D33" s="94"/>
-      <c r="E33" s="95"/>
-      <c r="F33" s="95"/>
-      <c r="G33" s="96"/>
+      <c r="D33" s="104"/>
+      <c r="E33" s="105"/>
+      <c r="F33" s="105"/>
+      <c r="G33" s="106"/>
       <c r="H33" s="34"/>
       <c r="I33" s="35"/>
       <c r="J33" s="6"/>
@@ -2489,10 +2298,10 @@
     <row r="34" spans="2:20" ht="30" customHeight="1">
       <c r="B34" s="8"/>
       <c r="C34" s="22"/>
-      <c r="D34" s="101"/>
-      <c r="E34" s="102"/>
-      <c r="F34" s="102"/>
-      <c r="G34" s="103"/>
+      <c r="D34" s="89"/>
+      <c r="E34" s="90"/>
+      <c r="F34" s="90"/>
+      <c r="G34" s="91"/>
       <c r="H34" s="46"/>
       <c r="I34" s="10"/>
       <c r="J34" s="9"/>
@@ -2823,8 +2632,8 @@
       </c>
     </row>
     <row r="51" spans="2:20" ht="14.25" customHeight="1" thickBot="1">
-      <c r="K51" s="104"/>
-      <c r="L51" s="104"/>
+      <c r="K51" s="92"/>
+      <c r="L51" s="92"/>
       <c r="T51" s="1" t="s">
         <v>52</v>
       </c>
@@ -2912,8 +2721,8 @@
       <c r="H55" s="84"/>
       <c r="I55" s="84"/>
       <c r="J55" s="84"/>
-      <c r="K55" s="100"/>
-      <c r="L55" s="100"/>
+      <c r="K55" s="88"/>
+      <c r="L55" s="88"/>
       <c r="M55" s="84"/>
       <c r="N55" s="84"/>
       <c r="O55" s="84"/>
@@ -2951,11 +2760,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="K55:L55"/>
-    <mergeCell ref="D34:G34"/>
-    <mergeCell ref="K51:L51"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="L32:N32"/>
     <mergeCell ref="B21:T21"/>
     <mergeCell ref="B22:T22"/>
     <mergeCell ref="O32:P32"/>
@@ -2965,6 +2769,11 @@
     <mergeCell ref="F26:G26"/>
     <mergeCell ref="F27:G27"/>
     <mergeCell ref="F28:G28"/>
+    <mergeCell ref="K55:L55"/>
+    <mergeCell ref="D34:G34"/>
+    <mergeCell ref="K51:L51"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="L32:N32"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>